<commit_message>
Updated Day 9 hotel to DREAM & HARMONY from updated Menalon trail Excel
</commit_message>
<xml_diff>
--- a/Menalon trail.xlsx
+++ b/Menalon trail.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6e4f9bd7d27fc20b/Documents/טיולים/יוון 10 2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="194" documentId="8_{5D33A2AF-B267-41C3-B7C1-67C7F3C3D1D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A466FCF6-B3E1-4740-801B-82FA9938B5B0}"/>
+  <xr:revisionPtr revIDLastSave="216" documentId="8_{5D33A2AF-B267-41C3-B7C1-67C7F3C3D1D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8E8B8B2-6CE2-47EE-B74D-BECDD599059B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{90CA65E1-AE0C-410C-A678-164840A6A514}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="104">
   <si>
     <t>מסלול</t>
   </si>
@@ -506,6 +506,75 @@
   </si>
   <si>
     <t>היום הארוך והמאתגר ביותר. מעבר בילאלי (Bilali Pass) מגיע לגובה של כ-1,550 מ'. מטיילים רבים ממליצים לקחת בבוקר מונית קצרה מדימיצאנה לזיגוביסטי (מקצר כ-4.2 ק"מ) כדי להפוך את היום ל-15 ק"מ נינוחים יותר. אלטי הוא כפר זעיר מאוד (כ-15 משפחות)</t>
+  </si>
+  <si>
+    <t>יום הליכה ותאריך</t>
+  </si>
+  <si>
+    <t>זמן נסיעה כולל להעברת הרכב</t>
+  </si>
+  <si>
+    <t>דימיצאנה (Dimitsana)</t>
+  </si>
+  <si>
+    <t>יום הליכה 1 (13/10)</t>
+  </si>
+  <si>
+    <t>אלטי (Elati)</t>
+  </si>
+  <si>
+    <t>יום הליכה 2 (14/10)</t>
+  </si>
+  <si>
+    <t>נימפאסיה (Nymfasia)</t>
+  </si>
+  <si>
+    <t>יום הליכה 3 (15/10)</t>
+  </si>
+  <si>
+    <t>ולטסיניקו (Valtesiniko)</t>
+  </si>
+  <si>
+    <t>יום הליכה 4 (16/10)</t>
+  </si>
+  <si>
+    <t>לגקאדיה (Lagkadia)</t>
+  </si>
+  <si>
+    <t>איסוף הרכב שנשאר בולטסיניקו</t>
+  </si>
+  <si>
+    <t>נקודת סיום מסלול ולינה</t>
+  </si>
+  <si>
+    <t>נקודת סיום מסלול למחרת</t>
+  </si>
+  <si>
+    <t>שעה ו-16 דקות (76 דק')(איסוף מסטמניצה + דילוג לאלטי + חזרה לדימיצאנה)</t>
+  </si>
+  <si>
+    <t>שעה ו-9 דקות (69 דק')(איסוף מדימיצאנה + דילוג לנימפאסיה + חזרה לאלטי)</t>
+  </si>
+  <si>
+    <t>שעה ו-8 דקות (68 דק')(איסוף מאלטי + דילוג לולטסיניקו + חזרה לנימפאסיה)</t>
+  </si>
+  <si>
+    <t>שעה ו-24 דקות (84 דק')(איסוף מנימפאסיה + דילוג ללגקאדיה + חזרה לולטסיניקו)</t>
+  </si>
+  <si>
+    <t>יום הליכה 5 (17/10)(סיום הטרק)</t>
+  </si>
+  <si>
+    <t>כ-56 דקות(לגקאדיה ← ולטסיניקו ← לגקאדיה)</t>
+  </si>
+  <si>
+    <t>DREAM &amp; HARMONY</t>
+  </si>
+  <si>
+    <t>ביטול 14/10. ללא ארוחת בוקר</t>
+  </si>
+  <si>
+    <t>Ktima Palivou, Nemea</t>
   </si>
 </sst>
 </file>
@@ -934,7 +1003,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5D788E2-AB74-4EDF-86AC-E682DB9A7C88}">
-  <dimension ref="A1:T11"/>
+  <dimension ref="A1:T19"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.296875" bestFit="1" customWidth="1"/>
@@ -1370,6 +1439,9 @@
       <c r="B8" t="s">
         <v>60</v>
       </c>
+      <c r="D8" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9">
@@ -1386,6 +1458,18 @@
       <c r="B10" t="s">
         <v>55</v>
       </c>
+      <c r="O10" t="s">
+        <v>101</v>
+      </c>
+      <c r="P10">
+        <v>79.8</v>
+      </c>
+      <c r="Q10">
+        <v>273</v>
+      </c>
+      <c r="R10" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11">
@@ -1396,6 +1480,90 @@
       </c>
       <c r="D11" t="s">
         <v>73</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B14" t="s">
+        <v>93</v>
+      </c>
+      <c r="C14" t="s">
+        <v>94</v>
+      </c>
+      <c r="D14" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>84</v>
+      </c>
+      <c r="B15" t="s">
+        <v>83</v>
+      </c>
+      <c r="C15" t="s">
+        <v>85</v>
+      </c>
+      <c r="D15" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" t="s">
+        <v>85</v>
+      </c>
+      <c r="C16" t="s">
+        <v>87</v>
+      </c>
+      <c r="D16" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>88</v>
+      </c>
+      <c r="B17" t="s">
+        <v>87</v>
+      </c>
+      <c r="C17" t="s">
+        <v>89</v>
+      </c>
+      <c r="D17" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>90</v>
+      </c>
+      <c r="B18" t="s">
+        <v>89</v>
+      </c>
+      <c r="C18" t="s">
+        <v>91</v>
+      </c>
+      <c r="D18" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>99</v>
+      </c>
+      <c r="B19" t="s">
+        <v>91</v>
+      </c>
+      <c r="C19" t="s">
+        <v>92</v>
+      </c>
+      <c r="D19" t="s">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>